<commit_message>
PAUSED (task146): strengthening (refusal recency), stage 4 next
The refiling share now depends on the region and on the month of the refusal:
in Western, Coastal and Island two thirds to nine tenths of a quarter's
last-month refusals file again in the next quarter's first claims week, under
one in five of its earlier months'. The third quarter's refusals there fell
55.3 per cent in September, so the call is 17,000 (16,895, one sigma 83);
regional sizing on the quarter taken whole files 15,000 (14,849, every
timing-blind construction 13,767 to 15,807), the national rate and the
seasonal route 13,000. The multiplicative form lands the golden's bin; leave
one turn out 303 against 635, 758, 880. No shipped sentence names recency,
timing or region (asserted); case-note withdrawal reasons varied. Checks 179,
verify agrees, two builds byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task146/golden/ic_preview_2026-10-10.xlsx
+++ b/task146/golden/ic_preview_2026-10-10.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>Initial claims preview, claims week ended 10 October 2026</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">  of which Western, Coastal and Island (%)</t>
   </si>
   <si>
+    <t xml:space="preserve">  of which Western, Coastal and Island, made in September (%)</t>
+  </si>
+  <si>
     <t>Claims expected to be filed again in the week, low</t>
   </si>
   <si>
@@ -61,7 +64,7 @@
     <t>The rest of the week, high</t>
   </si>
   <si>
-    <t>Each region's July to September determinations at the share its own first claims weeks of a quarter have filed again since 2014; about four fifths of the claims filed again are in Western, Coastal and Island.</t>
+    <t>Each region's July, August and September determinations, month by month, at the shares its own first claims weeks of a quarter have filed again since 2014; about nine tenths of the claims filed again are in Western, Coastal and Island.</t>
   </si>
   <si>
     <t>Workers to be laid off under layoff notices given to the board, by region of the site and month of the first layoff</t>
@@ -599,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A054BD3-0CA3-5D5A-B473-77AF429E572E}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="84.7109375" customWidth="1"/>
@@ -621,7 +624,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>16000</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -629,7 +632,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>11695</v>
+        <v>11814</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -642,7 +645,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="3">
-        <v>30182</v>
+        <v>26035</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -650,15 +653,15 @@
         <v>6</v>
       </c>
       <c r="B9" s="5">
-        <v>48.5</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="3">
-        <v>4000</v>
+      <c r="B10" s="5">
+        <v>55.3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -674,7 +677,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="3">
-        <v>11000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -682,12 +685,20 @@
         <v>10</v>
       </c>
       <c r="B13" s="3">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3">
         <v>12000</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -708,31 +719,31 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3">
         <v>111</v>
@@ -746,7 +757,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="3">
         <v>360</v>
@@ -760,7 +771,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="3">
         <v>205</v>
@@ -774,7 +785,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="3">
         <v>198</v>
@@ -788,7 +799,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="3">
         <v>198</v>
@@ -802,7 +813,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="3">
         <v>136</v>
@@ -816,7 +827,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="3">
         <v>300</v>
@@ -830,7 +841,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" s="3">
         <v>350</v>
@@ -844,7 +855,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="10">
         <v>1858</v>
@@ -874,236 +885,236 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3">
-        <v>7096</v>
+        <v>7094</v>
       </c>
       <c r="C5" s="3">
-        <v>7353</v>
+        <v>7554</v>
       </c>
       <c r="D5" s="5">
-        <v>3.6</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="3">
-        <v>3751</v>
+        <v>3725</v>
       </c>
       <c r="C6" s="3">
-        <v>3799</v>
+        <v>3759</v>
       </c>
       <c r="D6" s="5">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="3">
-        <v>21906</v>
+        <v>22193</v>
       </c>
       <c r="C7" s="3">
-        <v>20858</v>
+        <v>21265</v>
       </c>
       <c r="D7" s="5">
-        <v>-4.8</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="3">
-        <v>21899</v>
+        <v>22080</v>
       </c>
       <c r="C8" s="3">
-        <v>34794</v>
+        <v>35395</v>
       </c>
       <c r="D8" s="5">
-        <v>58.9</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="3">
-        <v>15444</v>
+        <v>15150</v>
       </c>
       <c r="C9" s="3">
-        <v>15565</v>
+        <v>15818</v>
       </c>
       <c r="D9" s="5">
-        <v>0.8</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3">
-        <v>15630</v>
+        <v>15482</v>
       </c>
       <c r="C10" s="3">
-        <v>15801</v>
+        <v>16114</v>
       </c>
       <c r="D10" s="5">
-        <v>1.1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" s="3">
-        <v>17623</v>
+        <v>17544</v>
       </c>
       <c r="C11" s="3">
-        <v>21427</v>
+        <v>22120</v>
       </c>
       <c r="D11" s="5">
-        <v>21.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="3">
-        <v>5130</v>
+        <v>5124</v>
       </c>
       <c r="C12" s="3">
         <v>4524</v>
       </c>
       <c r="D12" s="5">
-        <v>-11.8</v>
+        <v>-11.7</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="3">
-        <v>5865</v>
+        <v>5565</v>
       </c>
       <c r="C13" s="3">
-        <v>5454</v>
+        <v>5497</v>
       </c>
       <c r="D13" s="5">
-        <v>-7</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="3">
-        <v>7404</v>
+        <v>7585</v>
       </c>
       <c r="C14" s="3">
-        <v>7227</v>
+        <v>7108</v>
       </c>
       <c r="D14" s="5">
-        <v>-2.4</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="3">
-        <v>11876</v>
+        <v>11963</v>
       </c>
       <c r="C15" s="3">
-        <v>12032</v>
+        <v>12237</v>
       </c>
       <c r="D15" s="5">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" s="3">
-        <v>4095</v>
+        <v>3960</v>
       </c>
       <c r="C16" s="3">
-        <v>4053</v>
+        <v>4226</v>
       </c>
       <c r="D16" s="5">
-        <v>-1</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="3">
-        <v>4753</v>
+        <v>4676</v>
       </c>
       <c r="C17" s="3">
-        <v>4885</v>
+        <v>4905</v>
       </c>
       <c r="D17" s="5">
-        <v>2.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="3">
-        <v>13466</v>
+        <v>13386</v>
       </c>
       <c r="C18" s="3">
-        <v>12779</v>
+        <v>13022</v>
       </c>
       <c r="D18" s="5">
-        <v>-5.1</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="10">
-        <v>155938</v>
+        <v>155527</v>
       </c>
       <c r="C19" s="10">
-        <v>170551</v>
+        <v>173544</v>
       </c>
       <c r="D19" s="11">
-        <v>9.4</v>
+        <v>11.6</v>
       </c>
     </row>
   </sheetData>
@@ -1122,50 +1133,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>